<commit_message>
Initial backend commit (cleaned)
</commit_message>
<xml_diff>
--- a/static/sample_documents/Bulk CV Upload Format.xlsx
+++ b/static/sample_documents/Bulk CV Upload Format.xlsx
@@ -1,42 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kaleb\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahmed\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2CCDE60E-BAA2-47EB-9F97-3C3E857439C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7B0F0BC-5E22-48B0-9E80-A16388EC7066}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bulk CV Upload Format" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="83">
   <si>
     <t>email</t>
   </si>
@@ -116,22 +105,10 @@
     <t>tiktok</t>
   </si>
   <si>
-    <t>address_country</t>
-  </si>
-  <si>
     <t>address_region</t>
   </si>
   <si>
     <t>address_city</t>
-  </si>
-  <si>
-    <t>address_sub_city</t>
-  </si>
-  <si>
-    <t>address_woreda</t>
-  </si>
-  <si>
-    <t>address_kebele</t>
   </si>
   <si>
     <t>address_po_box</t>
@@ -303,7 +280,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1171,54 +1148,54 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AO9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:AO12"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.5703125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="30.54296875" style="1" customWidth="1"/>
     <col min="2" max="2" width="38" style="1" customWidth="1"/>
-    <col min="3" max="3" width="27.42578125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="27.453125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="19.7265625" style="1" customWidth="1"/>
     <col min="5" max="5" width="27" style="1" customWidth="1"/>
-    <col min="6" max="6" width="33.85546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="33.81640625" style="1" customWidth="1"/>
     <col min="7" max="7" width="15" style="1" customWidth="1"/>
-    <col min="8" max="8" width="19.140625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="19.1796875" style="2" customWidth="1"/>
     <col min="9" max="9" width="16" style="1" customWidth="1"/>
-    <col min="10" max="10" width="18.28515625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14.140625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="14.7109375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="18.5703125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="18.42578125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="22.85546875" style="1" customWidth="1"/>
-    <col min="16" max="16" width="25.42578125" style="1" customWidth="1"/>
-    <col min="17" max="17" width="25.5703125" style="1" customWidth="1"/>
-    <col min="18" max="18" width="16.85546875" style="1" customWidth="1"/>
-    <col min="19" max="19" width="17.140625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" style="1" customWidth="1"/>
-    <col min="21" max="21" width="25.28515625" style="1" customWidth="1"/>
-    <col min="22" max="22" width="17.28515625" style="1" customWidth="1"/>
-    <col min="23" max="23" width="13.140625" style="1" customWidth="1"/>
-    <col min="24" max="24" width="11.85546875" style="1" customWidth="1"/>
-    <col min="25" max="25" width="12.42578125" style="1" customWidth="1"/>
-    <col min="26" max="26" width="12.28515625" style="1" customWidth="1"/>
-    <col min="27" max="27" width="27.7109375" style="1" customWidth="1"/>
-    <col min="28" max="28" width="25.140625" style="1" customWidth="1"/>
-    <col min="29" max="29" width="24.7109375" style="1" customWidth="1"/>
-    <col min="30" max="30" width="28.7109375" style="1" customWidth="1"/>
-    <col min="31" max="31" width="23.5703125" style="1" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="1" customWidth="1"/>
-    <col min="33" max="33" width="16.5703125" style="1" customWidth="1"/>
-    <col min="34" max="34" width="17.85546875" style="1" customWidth="1"/>
-    <col min="35" max="35" width="21.85546875" style="1" customWidth="1"/>
-    <col min="36" max="36" width="20.42578125" style="1" customWidth="1"/>
-    <col min="37" max="37" width="19.140625" style="1" customWidth="1"/>
-    <col min="38" max="38" width="27.5703125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="18.26953125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="14.1796875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="14.7265625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="18.54296875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="18.453125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="22.81640625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="25.453125" style="1" customWidth="1"/>
+    <col min="17" max="17" width="25.54296875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="16.81640625" style="1" customWidth="1"/>
+    <col min="19" max="19" width="17.1796875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7265625" style="1" customWidth="1"/>
+    <col min="21" max="21" width="25.26953125" style="1" customWidth="1"/>
+    <col min="22" max="22" width="17.26953125" style="1" customWidth="1"/>
+    <col min="23" max="23" width="13.1796875" style="1" customWidth="1"/>
+    <col min="24" max="24" width="11.81640625" style="1" customWidth="1"/>
+    <col min="25" max="25" width="12.453125" style="1" customWidth="1"/>
+    <col min="26" max="26" width="12.26953125" style="1" customWidth="1"/>
+    <col min="27" max="27" width="27.7265625" style="1" customWidth="1"/>
+    <col min="28" max="28" width="25.1796875" style="1" customWidth="1"/>
+    <col min="29" max="29" width="24.7265625" style="1" customWidth="1"/>
+    <col min="30" max="30" width="28.7265625" style="1" customWidth="1"/>
+    <col min="31" max="31" width="23.54296875" style="1" customWidth="1"/>
+    <col min="32" max="32" width="14.7265625" style="1" customWidth="1"/>
+    <col min="33" max="33" width="16.54296875" style="1" customWidth="1"/>
+    <col min="34" max="34" width="17.81640625" style="1" customWidth="1"/>
+    <col min="35" max="35" width="21.81640625" style="1" customWidth="1"/>
+    <col min="36" max="36" width="20.453125" style="1" customWidth="1"/>
+    <col min="37" max="37" width="19.1796875" style="1" customWidth="1"/>
+    <col min="38" max="38" width="27.54296875" style="1" customWidth="1"/>
     <col min="39" max="39" width="31" style="1" customWidth="1"/>
-    <col min="40" max="40" width="20.85546875" style="1" customWidth="1"/>
-    <col min="41" max="41" width="8.85546875" style="1"/>
-    <col min="42" max="16384" width="9.140625" style="3"/>
+    <col min="40" max="40" width="20.81640625" style="1" customWidth="1"/>
+    <col min="41" max="41" width="8.81640625" style="1"/>
+    <col min="42" max="16384" width="9.1796875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40">
+    <row r="1" spans="1:41" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1327,43 +1304,35 @@
       <c r="AJ1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="3"/>
+      <c r="AM1" s="3"/>
+      <c r="AN1" s="3"/>
+      <c r="AO1" s="3"/>
+    </row>
+    <row r="2" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AN1" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="2" spans="1:40" ht="16.5">
-      <c r="A2" s="4" t="s">
-        <v>40</v>
       </c>
       <c r="B2" s="1">
         <v>343434</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="H2" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>46</v>
       </c>
       <c r="I2" s="1">
         <v>3</v>
@@ -1372,66 +1341,70 @@
         <v>5</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="L2" s="5">
         <v>45749</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="Q2" s="1">
         <v>3</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="S2" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="T2" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="AG2" s="1">
+        <v>47</v>
+      </c>
+      <c r="AC2" s="1">
         <v>200</v>
       </c>
-      <c r="AL2" s="1" t="s">
-        <v>52</v>
-      </c>
+      <c r="AH2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AL2" s="3"/>
+      <c r="AM2" s="3"/>
+      <c r="AN2" s="3"/>
+      <c r="AO2" s="3"/>
     </row>
-    <row r="3" spans="1:40" ht="16.5">
+    <row r="3" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B3" s="6">
         <v>343434</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="I3" s="1">
         <v>3</v>
@@ -1440,66 +1413,70 @@
         <v>5</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="L3" s="5">
         <v>45750</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="Q3" s="1">
         <v>4</v>
       </c>
       <c r="R3" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="S3" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="T3" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="AG3" s="1">
+        <v>47</v>
+      </c>
+      <c r="AC3" s="1">
         <v>201</v>
       </c>
-      <c r="AL3" s="1" t="s">
-        <v>58</v>
-      </c>
+      <c r="AH3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL3" s="3"/>
+      <c r="AM3" s="3"/>
+      <c r="AN3" s="3"/>
+      <c r="AO3" s="3"/>
     </row>
-    <row r="4" spans="1:40" ht="16.5">
+    <row r="4" spans="1:41" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B4" s="6">
         <v>343435</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I4" s="1">
         <v>3</v>
@@ -1508,66 +1485,70 @@
         <v>5</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="L4" s="5">
         <v>45751</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="Q4" s="1">
         <v>5</v>
       </c>
       <c r="R4" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="S4" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="AG4" s="1">
+        <v>47</v>
+      </c>
+      <c r="AC4" s="1">
         <v>202</v>
       </c>
-      <c r="AL4" s="1" t="s">
-        <v>64</v>
-      </c>
+      <c r="AH4" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL4" s="3"/>
+      <c r="AM4" s="3"/>
+      <c r="AN4" s="3"/>
+      <c r="AO4" s="3"/>
     </row>
-    <row r="5" spans="1:40" ht="16.5">
+    <row r="5" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B5" s="6">
         <v>343436</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="I5" s="1">
         <v>3</v>
@@ -1576,66 +1557,70 @@
         <v>5</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="L5" s="5">
         <v>45752</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="Q5" s="1">
         <v>6</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="S5" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="T5" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="AG5" s="1">
+        <v>47</v>
+      </c>
+      <c r="AC5" s="1">
         <v>203</v>
       </c>
-      <c r="AL5" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="AH5" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL5" s="3"/>
+      <c r="AM5" s="3"/>
+      <c r="AN5" s="3"/>
+      <c r="AO5" s="3"/>
     </row>
-    <row r="6" spans="1:40" ht="16.5">
+    <row r="6" spans="1:41" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B6" s="6">
         <v>343437</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="I6" s="1">
         <v>3</v>
@@ -1644,66 +1629,70 @@
         <v>5</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="L6" s="5">
         <v>45753</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q6" s="1">
         <v>7</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="S6" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="T6" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="AG6" s="1">
+        <v>47</v>
+      </c>
+      <c r="AC6" s="1">
         <v>204</v>
       </c>
-      <c r="AL6" s="1" t="s">
-        <v>74</v>
-      </c>
+      <c r="AH6" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL6" s="3"/>
+      <c r="AM6" s="3"/>
+      <c r="AN6" s="3"/>
+      <c r="AO6" s="3"/>
     </row>
-    <row r="7" spans="1:40" ht="16.5">
+    <row r="7" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6">
         <v>343438</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="I7" s="1">
         <v>3</v>
@@ -1712,66 +1701,70 @@
         <v>5</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="L7" s="5">
         <v>45754</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="Q7" s="1">
         <v>8</v>
       </c>
       <c r="R7" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="S7" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="T7" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="AG7" s="1">
+        <v>47</v>
+      </c>
+      <c r="AC7" s="1">
         <v>205</v>
       </c>
-      <c r="AL7" s="1" t="s">
-        <v>78</v>
-      </c>
+      <c r="AH7" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="AL7" s="3"/>
+      <c r="AM7" s="3"/>
+      <c r="AN7" s="3"/>
+      <c r="AO7" s="3"/>
     </row>
-    <row r="8" spans="1:40" ht="16.5">
+    <row r="8" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B8" s="6">
         <v>343439</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="I8" s="1">
         <v>3</v>
@@ -1780,66 +1773,70 @@
         <v>5</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="L8" s="5">
         <v>45755</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="Q8" s="1">
         <v>9</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="AG8" s="1">
+        <v>47</v>
+      </c>
+      <c r="AC8" s="1">
         <v>206</v>
       </c>
-      <c r="AL8" s="1" t="s">
-        <v>82</v>
-      </c>
+      <c r="AH8" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="AL8" s="3"/>
+      <c r="AM8" s="3"/>
+      <c r="AN8" s="3"/>
+      <c r="AO8" s="3"/>
     </row>
-    <row r="9" spans="1:40" ht="16.5">
+    <row r="9" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B9" s="6">
         <v>343440</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="I9" s="1">
         <v>3</v>
@@ -1848,41 +1845,57 @@
         <v>5</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="L9" s="5">
         <v>45756</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="Q9" s="1">
         <v>10</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="AG9" s="1">
+        <v>47</v>
+      </c>
+      <c r="AC9" s="1">
         <v>207</v>
       </c>
-      <c r="AL9" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="AH9" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="AL9" s="3"/>
+      <c r="AM9" s="3"/>
+      <c r="AN9" s="3"/>
+      <c r="AO9" s="3"/>
+    </row>
+    <row r="10" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="AL10" s="3"/>
+      <c r="AM10" s="3"/>
+      <c r="AN10" s="3"/>
+      <c r="AO10" s="3"/>
+    </row>
+    <row r="11" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="AO11" s="3"/>
+    </row>
+    <row r="12" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="AO12" s="3"/>
     </row>
   </sheetData>
   <dataValidations count="5">
@@ -1898,7 +1911,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K1:K1048576" xr:uid="{232DA69C-D4CA-4DA8-924A-9B10F6C59D96}">
       <formula1>"very_light, light, medium, dark, very_dark"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AL1:AL1048576" xr:uid="{FBD3B295-E821-419A-8EA7-38B10E81D465}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH1:AH10 AK11:AK12 AL13:AL1048576" xr:uid="{FBD3B295-E821-419A-8EA7-38B10E81D465}">
       <formula1>" no_education, primary_education, secondary_education, vocational, some_college_courses, bsc, msc, phd"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>